<commit_message>
chore: replace the Axiometrics citations in synthetic fixtures
The Oakwood underwriting workbooks and the draft IC memo cited
"Axiometrics" (a real market-data provider) as the source of the 3.8%
rent growth figure. They now cite a "Synthetic Rent Survey". The three
workbooks were edited in place at the XML level, so every other part of
each file is byte-identical, and the extractor snapshot for the one
workbook in the demo set was regenerated with
services/extractor/scripts/snapshot_fixtures.py (text and sha256 only).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/synthetic-capital/Fund II - Synthetic Value Fund II/Oakwood_Commons/acquisition/UW_OakwoodCommons_v3_AD_112020.xlsx
+++ b/fixtures/synthetic-capital/Fund II - Synthetic Value Fund II/Oakwood_Commons/acquisition/UW_OakwoodCommons_v3_AD_112020.xlsx
@@ -640,7 +640,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PN using 2.5% rent growth is too conservative — see Axiometrics data in comps tab, Houston submarket running 3.8% trailing 12.</v>
+        <v>PN using 2.5% rent growth is too conservative — see Synthetic Rent Survey data in comps tab, Houston submarket running 3.8% trailing 12.</v>
       </c>
     </row>
     <row r="35">
@@ -822,7 +822,7 @@
         <v>annual</v>
       </c>
       <c r="D15" t="str">
-        <v>Axiometrics shows 3.8% trailing</v>
+        <v>Synthetic Rent Survey shows 3.8% trailing</v>
       </c>
     </row>
     <row r="16">
@@ -2354,7 +2354,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>AXIOMETRICS MARKET DATA</v>
+        <v>SYNTHETIC RENT SURVEY MARKET DATA</v>
       </c>
     </row>
     <row r="10">

</xml_diff>